<commit_message>
fix(plan-pizzeria): revisión final aplicada (1 B · 8 M · 15 m) — gates F2 en verde
B1 Instrucciones ya no manda el coste de una pizza a Supuestos!B13 · M1 {PAYBACK} legible con cualquier valor ·
M2 «con azúcares o edulcorantes añadidos» (LIVA 91.Uno.1.1.º b) · M3-M8 coherencia calculadora/Excel/Word/landing ·
guarda RX_PUBLICA contra la trampa de motor.TILDES. Detalle en plan-pizzeria/REVISION-FINAL.md.

Via: Claude Code

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/plan-negocio-pizzeria/calculadora-masa-escandallo-pizzeria.xlsx
+++ b/astro-site/public/dl/plan-negocio-pizzeria/calculadora-masa-escandallo-pizzeria.xlsx
@@ -712,7 +712,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Pliego: hasta 1.800 g de harina por litro de agua («punto de amasado»). El mínimo de 1.600 g es el que da una absorción del 62 % (cálculo del kit sobre el rango de 55-62 % del pliego).</t>
+          <t>El pliego solo fija el máximo: hasta 1.800 g de harina por litro de agua («punto de amasado»). El mínimo de 1.600 g (62,5 % de hidratación) es un cálculo del kit sobre la absorción de 55-62 % que el pliego pide a la harina.</t>
         </is>
       </c>
     </row>
@@ -1383,7 +1383,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Comida preparada, en sala, para llevar y a domicilio: 10 % (Ley 37/1992, art. 91.Uno.2.2.º).</t>
+          <t>Comida preparada, en sala, para llevar y a domicilio: 10 % (Ley 37/1992, art. 91.Uno.1.1.º y 2.2.º).</t>
         </is>
       </c>
     </row>
@@ -3209,7 +3209,7 @@
     <row r="21" ht="45" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>El IVA de la comida preparada para consumir en el local, para llevar o a domicilio es el 10 % (Ley 37/1992, art. 91.Uno.2.2.º). Las bebidas alcohólicas y los refrescos con azúcar que salen del local llevan el 21 % y no están en este escandallo.</t>
+          <t>El IVA de la comida preparada para consumir en el local, para llevar o a domicilio es el 10 % (Ley 37/1992, art. 91.Uno.1.1.º y 2.2.º). Las bebidas alcohólicas y los refrescos con azúcares o edulcorantes añadidos que salen del local llevan el 21 % y no están en este escandallo.</t>
         </is>
       </c>
     </row>

</xml_diff>